<commit_message>
Update content two files: index.html and file html/page1.html
</commit_message>
<xml_diff>
--- a/DA24TTC-To2.xlsx
+++ b/DA24TTC-To2.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="103">
   <si>
     <t>Đại học Trà Vinh</t>
   </si>
@@ -96,9 +96,6 @@
     <t>1</t>
   </si>
   <si>
-    <t>110124063</t>
-  </si>
-  <si>
     <t>Dương Thành</t>
   </si>
   <si>
@@ -168,18 +165,12 @@
     <t>7</t>
   </si>
   <si>
-    <t>110124088</t>
-  </si>
-  <si>
     <t>Nguyễn Hoài</t>
   </si>
   <si>
     <t>8</t>
   </si>
   <si>
-    <t>110124094</t>
-  </si>
-  <si>
     <t>Trần Thiện</t>
   </si>
   <si>
@@ -213,9 +204,6 @@
     <t>11</t>
   </si>
   <si>
-    <t>110124114</t>
-  </si>
-  <si>
     <t>Nguyễn Thị Lưu</t>
   </si>
   <si>
@@ -225,9 +213,6 @@
     <t>12</t>
   </si>
   <si>
-    <t>110124115</t>
-  </si>
-  <si>
     <t>Trần Thị Trúc</t>
   </si>
   <si>
@@ -249,18 +234,12 @@
     <t>14</t>
   </si>
   <si>
-    <t>110124121</t>
-  </si>
-  <si>
     <t>Trần Khải</t>
   </si>
   <si>
     <t>15</t>
   </si>
   <si>
-    <t>110124242</t>
-  </si>
-  <si>
     <t>Nguyễn Hoàng</t>
   </si>
   <si>
@@ -270,9 +249,6 @@
     <t>16</t>
   </si>
   <si>
-    <t>110124244</t>
-  </si>
-  <si>
     <t>Huỳnh Thị Kim</t>
   </si>
   <si>
@@ -282,9 +258,6 @@
     <t>17</t>
   </si>
   <si>
-    <t>110124246</t>
-  </si>
-  <si>
     <t>Tăng Kiều</t>
   </si>
   <si>
@@ -292,9 +265,6 @@
   </si>
   <si>
     <t>18</t>
-  </si>
-  <si>
-    <t>110124247</t>
   </si>
   <si>
     <t>Võ Thị Thảo</t>
@@ -357,6 +327,9 @@
   <si>
     <t>Bài 2
 Quản lý dự án với Github</t>
+  </si>
+  <si>
+    <t>Hỗ trợ bạn</t>
   </si>
 </sst>
 </file>
@@ -456,7 +429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -475,6 +448,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -816,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
@@ -826,46 +809,48 @@
     <col min="5" max="5" width="15.85546875" customWidth="1"/>
     <col min="6" max="6" width="50.85546875" customWidth="1"/>
     <col min="7" max="8" width="15.85546875" customWidth="1"/>
-    <col min="9" max="9" width="30.85546875" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" style="5" customWidth="1"/>
+    <col min="10" max="10" width="30.85546875" customWidth="1"/>
+    <col min="11" max="11" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:11">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="G1" s="5" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="G1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="5"/>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="5" t="s">
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="G2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="5"/>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="D4" s="5" t="s">
+      <c r="H2" s="8"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="D4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="D5" s="5" t="s">
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="D5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-    </row>
-    <row r="7" spans="1:9">
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+    </row>
+    <row r="7" spans="1:11">
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -879,7 +864,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:11">
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
@@ -893,7 +878,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:11">
       <c r="B9" s="1" t="s">
         <v>14</v>
       </c>
@@ -907,7 +892,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="42.75">
+    <row r="11" spans="1:11" ht="42.75">
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
@@ -927,541 +912,629 @@
         <v>23</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+        <v>100</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K11" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="3">
+        <v>110124063</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>27</v>
-      </c>
       <c r="E12" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3">
         <v>10</v>
       </c>
-      <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="1:9">
+      <c r="I12" s="10"/>
+      <c r="J12" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="D13" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G13" s="3">
         <v>4</v>
       </c>
       <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-    </row>
-    <row r="14" spans="1:9">
+      <c r="I13" s="10"/>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>35</v>
-      </c>
       <c r="E14" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G14" s="3">
         <v>4</v>
       </c>
       <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-    </row>
-    <row r="15" spans="1:9">
+      <c r="I14" s="10"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>39</v>
-      </c>
       <c r="E15" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3">
         <v>12</v>
       </c>
-      <c r="I15" s="3"/>
-    </row>
-    <row r="16" spans="1:9">
+      <c r="I15" s="10"/>
+      <c r="J15" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="E16" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3">
         <v>10</v>
       </c>
-      <c r="I16" s="3"/>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="I16" s="10"/>
+      <c r="J16" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="E17" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G17" s="3">
         <v>4</v>
       </c>
       <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-    </row>
-    <row r="18" spans="1:9">
+      <c r="I17" s="10"/>
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" spans="1:11">
       <c r="A18" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="3">
+        <v>110124088</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>50</v>
-      </c>
       <c r="D18" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3">
         <v>12</v>
       </c>
-      <c r="I18" s="3"/>
-    </row>
-    <row r="19" spans="1:9">
+      <c r="I18" s="10">
+        <v>110124115</v>
+      </c>
+      <c r="J18" s="3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="3">
+        <v>110124094</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>54</v>
-      </c>
       <c r="E19" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3">
         <v>16</v>
       </c>
-      <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="1:9">
+      <c r="I19" s="10">
+        <v>110124063</v>
+      </c>
+      <c r="J19" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>58</v>
-      </c>
       <c r="E20" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="3">
         <v>14</v>
       </c>
-      <c r="I20" s="3"/>
-    </row>
-    <row r="21" spans="1:9">
+      <c r="I20" s="10">
+        <v>110124242</v>
+      </c>
+      <c r="J20" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>62</v>
-      </c>
       <c r="E21" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="H21" s="3">
         <v>18</v>
       </c>
-      <c r="I21" s="3"/>
-    </row>
-    <row r="22" spans="1:9">
+      <c r="I21" s="10">
+        <v>110124063</v>
+      </c>
+      <c r="J21" s="3">
+        <v>44</v>
+      </c>
+      <c r="K21" s="5">
+        <v>110124247</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
       <c r="A22" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
+      </c>
+      <c r="B22" s="3">
+        <v>110124114</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3">
         <v>14</v>
       </c>
-      <c r="I22" s="3"/>
-    </row>
-    <row r="23" spans="1:9">
+      <c r="I22" s="10">
+        <v>110124244</v>
+      </c>
+      <c r="J22" s="3">
+        <v>48</v>
+      </c>
+      <c r="K22" s="5">
+        <v>110124247</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>68</v>
+        <v>63</v>
+      </c>
+      <c r="B23" s="3">
+        <v>110124115</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="3">
         <v>10</v>
       </c>
-      <c r="I23" s="3"/>
-    </row>
-    <row r="24" spans="1:9">
+      <c r="I23" s="10"/>
+      <c r="J23" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
       <c r="A24" s="3" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3">
         <v>20</v>
       </c>
-      <c r="I24" s="3"/>
-    </row>
-    <row r="25" spans="1:9">
+      <c r="I24" s="10">
+        <v>110124114</v>
+      </c>
+      <c r="J24" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
       <c r="A25" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>76</v>
+        <v>70</v>
+      </c>
+      <c r="B25" s="3">
+        <v>110124121</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3">
         <v>11</v>
       </c>
-      <c r="I25" s="3"/>
-    </row>
-    <row r="26" spans="1:9">
+      <c r="I25" s="10">
+        <v>110124244</v>
+      </c>
+      <c r="J25" s="3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
       <c r="A26" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>79</v>
+        <v>72</v>
+      </c>
+      <c r="B26" s="3">
+        <v>110124242</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3">
         <v>12</v>
       </c>
-      <c r="I26" s="3"/>
-    </row>
-    <row r="27" spans="1:9">
+      <c r="I26" s="10"/>
+      <c r="J26" s="3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
       <c r="A27" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>83</v>
+        <v>75</v>
+      </c>
+      <c r="B27" s="3">
+        <v>110124244</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="7">
         <v>8</v>
       </c>
-      <c r="I27" s="3"/>
-    </row>
-    <row r="28" spans="1:9">
+      <c r="I27" s="11"/>
+      <c r="J27" s="3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
       <c r="A28" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>87</v>
+        <v>78</v>
+      </c>
+      <c r="B28" s="3">
+        <v>110124246</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3">
         <v>11</v>
       </c>
-      <c r="I28" s="3"/>
-    </row>
-    <row r="29" spans="1:9">
+      <c r="I28" s="10"/>
+      <c r="J28" s="3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
       <c r="A29" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>91</v>
+        <v>81</v>
+      </c>
+      <c r="B29" s="3">
+        <v>110124247</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="3">
         <v>11</v>
       </c>
-      <c r="I29" s="3"/>
-    </row>
-    <row r="30" spans="1:9">
+      <c r="I29" s="10"/>
+      <c r="J29" s="3">
+        <v>27</v>
+      </c>
+      <c r="K29" s="5">
+        <v>110124121</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
       <c r="A30" s="3" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3">
         <v>11</v>
       </c>
-      <c r="I30" s="3"/>
-    </row>
-    <row r="31" spans="1:9">
+      <c r="I30" s="10">
+        <v>110124247</v>
+      </c>
+      <c r="J30" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
       <c r="A31" s="3" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="G31" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
-    </row>
-    <row r="32" spans="1:9">
+      <c r="I31" s="10"/>
+      <c r="J31" s="3"/>
+    </row>
+    <row r="32" spans="1:11">
       <c r="A32" s="3" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G32" s="3"/>
       <c r="H32" s="3">
         <v>15</v>
       </c>
-      <c r="I32" s="3"/>
+      <c r="I32" s="10">
+        <v>110124242</v>
+      </c>
+      <c r="J32" s="3">
+        <v>41</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1474,7 +1547,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I10 A12:F32 A11:F11" numberStoredAsText="1"/>
+    <ignoredError sqref="J1:J10 A11:F11 A1:H10 A20:F21 A19 C19:F19 A13:F17 A12 C12:F12 A18 C18:F18 A24:F24 A22 C22:F22 A30:F32 A26 C26:F26 A27 C27:F27 A28 C28:F28 A29 C29:F29 A23 C23:F23 A25 C25:F25" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>